<commit_message>
wip: dropdown alignment and csv export features
</commit_message>
<xml_diff>
--- a/tomorrowcities/assets/data/sample_scenario_input/3_household.xlsx
+++ b/tomorrowcities/assets/data/sample_scenario_input/3_household.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eo\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eo\Desktop\tomorrowscities\tomorrowcities\assets\data\sample_scenario_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E32C2B3D-1EFA-4673-A752-837228BC0080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D290D99C-A44F-4238-9FC0-47525B07171C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31800" yWindow="2115" windowWidth="22905" windowHeight="12810" xr2:uid="{CB7973E4-52BA-43C8-A4DC-03E2712D70C0}"/>
+    <workbookView xWindow="2355" yWindow="750" windowWidth="24255" windowHeight="13800" xr2:uid="{CB7973E4-52BA-43C8-A4DC-03E2712D70C0}"/>
   </bookViews>
   <sheets>
     <sheet name="3_household" sheetId="1" r:id="rId1"/>
@@ -37,13 +37,13 @@
     <t>commfacid</t>
   </si>
   <si>
-    <t>lowIncomeA</t>
-  </si>
-  <si>
     <t>midIncome</t>
   </si>
   <si>
-    <t>lowIncomeB</t>
+    <t>veryLowIncome</t>
+  </si>
+  <si>
+    <t>lowIncome</t>
   </si>
 </sst>
 </file>
@@ -886,6 +886,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9B6BA27-2DE6-481C-BCA8-AAA0C737D574}">
   <dimension ref="A1:E371"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="33" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -912,7 +915,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -929,7 +932,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3">
         <v>4</v>
@@ -946,7 +949,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -963,7 +966,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -980,7 +983,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -997,7 +1000,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -1014,7 +1017,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8">
         <v>3</v>
@@ -1031,7 +1034,7 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9">
         <v>3</v>
@@ -1048,7 +1051,7 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1065,7 +1068,7 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D11">
         <v>4</v>
@@ -1082,7 +1085,7 @@
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12">
         <v>4</v>
@@ -1099,7 +1102,7 @@
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -1116,7 +1119,7 @@
         <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D14">
         <v>3</v>
@@ -1133,7 +1136,7 @@
         <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -1150,7 +1153,7 @@
         <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D16">
         <v>4</v>
@@ -1167,7 +1170,7 @@
         <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -1184,7 +1187,7 @@
         <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D18">
         <v>3</v>
@@ -1201,7 +1204,7 @@
         <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -1218,7 +1221,7 @@
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D20">
         <v>4</v>
@@ -1235,7 +1238,7 @@
         <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D21">
         <v>4</v>
@@ -1252,7 +1255,7 @@
         <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -1269,7 +1272,7 @@
         <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1286,7 +1289,7 @@
         <v>39</v>
       </c>
       <c r="C24" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D24">
         <v>4</v>
@@ -1303,7 +1306,7 @@
         <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -1320,7 +1323,7 @@
         <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D26">
         <v>4</v>
@@ -1337,7 +1340,7 @@
         <v>42</v>
       </c>
       <c r="C27" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D27">
         <v>2</v>
@@ -1354,7 +1357,7 @@
         <v>43</v>
       </c>
       <c r="C28" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D28">
         <v>3</v>
@@ -1371,7 +1374,7 @@
         <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D29">
         <v>2</v>
@@ -1388,7 +1391,7 @@
         <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D30">
         <v>4</v>
@@ -1405,7 +1408,7 @@
         <v>55</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D31">
         <v>2</v>
@@ -1422,7 +1425,7 @@
         <v>56</v>
       </c>
       <c r="C32" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D32">
         <v>4</v>
@@ -1439,7 +1442,7 @@
         <v>57</v>
       </c>
       <c r="C33" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D33">
         <v>2</v>
@@ -1456,7 +1459,7 @@
         <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D34">
         <v>3</v>
@@ -1473,7 +1476,7 @@
         <v>59</v>
       </c>
       <c r="C35" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D35">
         <v>2</v>
@@ -1490,7 +1493,7 @@
         <v>61</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D36">
         <v>3</v>
@@ -1507,7 +1510,7 @@
         <v>62</v>
       </c>
       <c r="C37" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -1524,7 +1527,7 @@
         <v>64</v>
       </c>
       <c r="C38" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D38">
         <v>4</v>
@@ -1541,7 +1544,7 @@
         <v>65</v>
       </c>
       <c r="C39" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -1558,7 +1561,7 @@
         <v>66</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -1575,7 +1578,7 @@
         <v>67</v>
       </c>
       <c r="C41" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D41">
         <v>2</v>
@@ -1592,7 +1595,7 @@
         <v>68</v>
       </c>
       <c r="C42" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D42">
         <v>3</v>
@@ -1609,7 +1612,7 @@
         <v>69</v>
       </c>
       <c r="C43" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D43">
         <v>3</v>
@@ -1626,7 +1629,7 @@
         <v>70</v>
       </c>
       <c r="C44" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -1643,7 +1646,7 @@
         <v>71</v>
       </c>
       <c r="C45" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D45">
         <v>2</v>
@@ -1660,7 +1663,7 @@
         <v>72</v>
       </c>
       <c r="C46" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D46">
         <v>3</v>
@@ -1677,7 +1680,7 @@
         <v>73</v>
       </c>
       <c r="C47" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D47">
         <v>4</v>
@@ -1694,7 +1697,7 @@
         <v>74</v>
       </c>
       <c r="C48" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D48">
         <v>2</v>
@@ -1711,7 +1714,7 @@
         <v>75</v>
       </c>
       <c r="C49" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D49">
         <v>2</v>
@@ -1728,7 +1731,7 @@
         <v>76</v>
       </c>
       <c r="C50" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D50">
         <v>4</v>
@@ -1745,7 +1748,7 @@
         <v>77</v>
       </c>
       <c r="C51" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D51">
         <v>3</v>
@@ -1762,7 +1765,7 @@
         <v>78</v>
       </c>
       <c r="C52" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D52">
         <v>3</v>
@@ -1779,7 +1782,7 @@
         <v>79</v>
       </c>
       <c r="C53" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D53">
         <v>2</v>
@@ -1796,7 +1799,7 @@
         <v>80</v>
       </c>
       <c r="C54" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D54">
         <v>3</v>
@@ -1813,7 +1816,7 @@
         <v>81</v>
       </c>
       <c r="C55" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D55">
         <v>3</v>
@@ -1830,7 +1833,7 @@
         <v>82</v>
       </c>
       <c r="C56" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D56">
         <v>3</v>
@@ -1847,7 +1850,7 @@
         <v>83</v>
       </c>
       <c r="C57" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D57">
         <v>4</v>
@@ -1864,7 +1867,7 @@
         <v>85</v>
       </c>
       <c r="C58" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D58">
         <v>4</v>
@@ -1881,7 +1884,7 @@
         <v>86</v>
       </c>
       <c r="C59" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D59">
         <v>4</v>
@@ -1898,7 +1901,7 @@
         <v>87</v>
       </c>
       <c r="C60" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D60">
         <v>4</v>
@@ -1915,7 +1918,7 @@
         <v>88</v>
       </c>
       <c r="C61" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -1932,7 +1935,7 @@
         <v>89</v>
       </c>
       <c r="C62" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -1949,7 +1952,7 @@
         <v>90</v>
       </c>
       <c r="C63" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D63">
         <v>3</v>
@@ -1966,7 +1969,7 @@
         <v>91</v>
       </c>
       <c r="C64" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D64">
         <v>3</v>
@@ -1983,7 +1986,7 @@
         <v>92</v>
       </c>
       <c r="C65" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D65">
         <v>2</v>
@@ -2000,7 +2003,7 @@
         <v>93</v>
       </c>
       <c r="C66" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D66">
         <v>2</v>
@@ -2017,7 +2020,7 @@
         <v>94</v>
       </c>
       <c r="C67" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D67">
         <v>4</v>
@@ -2034,7 +2037,7 @@
         <v>95</v>
       </c>
       <c r="C68" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D68">
         <v>2</v>
@@ -2051,7 +2054,7 @@
         <v>96</v>
       </c>
       <c r="C69" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D69">
         <v>4</v>
@@ -2068,7 +2071,7 @@
         <v>97</v>
       </c>
       <c r="C70" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D70">
         <v>1</v>
@@ -2085,7 +2088,7 @@
         <v>98</v>
       </c>
       <c r="C71" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D71">
         <v>4</v>
@@ -2102,7 +2105,7 @@
         <v>99</v>
       </c>
       <c r="C72" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D72">
         <v>1</v>
@@ -2119,7 +2122,7 @@
         <v>100</v>
       </c>
       <c r="C73" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D73">
         <v>4</v>
@@ -2136,7 +2139,7 @@
         <v>101</v>
       </c>
       <c r="C74" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D74">
         <v>2</v>
@@ -2153,7 +2156,7 @@
         <v>102</v>
       </c>
       <c r="C75" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D75">
         <v>4</v>
@@ -2170,7 +2173,7 @@
         <v>103</v>
       </c>
       <c r="C76" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D76">
         <v>3</v>
@@ -2187,7 +2190,7 @@
         <v>104</v>
       </c>
       <c r="C77" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D77">
         <v>2</v>
@@ -2204,7 +2207,7 @@
         <v>105</v>
       </c>
       <c r="C78" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D78">
         <v>4</v>
@@ -2221,7 +2224,7 @@
         <v>106</v>
       </c>
       <c r="C79" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D79">
         <v>2</v>
@@ -2238,7 +2241,7 @@
         <v>107</v>
       </c>
       <c r="C80" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D80">
         <v>3</v>
@@ -2255,7 +2258,7 @@
         <v>108</v>
       </c>
       <c r="C81" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D81">
         <v>4</v>
@@ -2272,7 +2275,7 @@
         <v>109</v>
       </c>
       <c r="C82" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D82">
         <v>1</v>
@@ -2289,7 +2292,7 @@
         <v>110</v>
       </c>
       <c r="C83" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D83">
         <v>3</v>
@@ -2306,7 +2309,7 @@
         <v>111</v>
       </c>
       <c r="C84" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D84">
         <v>4</v>
@@ -2323,7 +2326,7 @@
         <v>112</v>
       </c>
       <c r="C85" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D85">
         <v>4</v>
@@ -2340,7 +2343,7 @@
         <v>113</v>
       </c>
       <c r="C86" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D86">
         <v>3</v>
@@ -2357,7 +2360,7 @@
         <v>114</v>
       </c>
       <c r="C87" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D87">
         <v>1</v>
@@ -2374,7 +2377,7 @@
         <v>125</v>
       </c>
       <c r="C88" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D88">
         <v>4</v>
@@ -2391,7 +2394,7 @@
         <v>126</v>
       </c>
       <c r="C89" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D89">
         <v>3</v>
@@ -2408,7 +2411,7 @@
         <v>128</v>
       </c>
       <c r="C90" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D90">
         <v>4</v>
@@ -2425,7 +2428,7 @@
         <v>129</v>
       </c>
       <c r="C91" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D91">
         <v>3</v>
@@ -2442,7 +2445,7 @@
         <v>130</v>
       </c>
       <c r="C92" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D92">
         <v>4</v>
@@ -2459,7 +2462,7 @@
         <v>132</v>
       </c>
       <c r="C93" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D93">
         <v>3</v>
@@ -2476,7 +2479,7 @@
         <v>133</v>
       </c>
       <c r="C94" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D94">
         <v>4</v>
@@ -2493,7 +2496,7 @@
         <v>134</v>
       </c>
       <c r="C95" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -2510,7 +2513,7 @@
         <v>135</v>
       </c>
       <c r="C96" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D96">
         <v>4</v>
@@ -2527,7 +2530,7 @@
         <v>136</v>
       </c>
       <c r="C97" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D97">
         <v>4</v>
@@ -2544,7 +2547,7 @@
         <v>137</v>
       </c>
       <c r="C98" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D98">
         <v>2</v>
@@ -2561,7 +2564,7 @@
         <v>139</v>
       </c>
       <c r="C99" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D99">
         <v>2</v>
@@ -2578,7 +2581,7 @@
         <v>151</v>
       </c>
       <c r="C100" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D100">
         <v>4</v>
@@ -2595,7 +2598,7 @@
         <v>152</v>
       </c>
       <c r="C101" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D101">
         <v>3</v>
@@ -2612,7 +2615,7 @@
         <v>153</v>
       </c>
       <c r="C102" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D102">
         <v>1</v>
@@ -2629,7 +2632,7 @@
         <v>154</v>
       </c>
       <c r="C103" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D103">
         <v>3</v>
@@ -2646,7 +2649,7 @@
         <v>155</v>
       </c>
       <c r="C104" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D104">
         <v>4</v>
@@ -2663,7 +2666,7 @@
         <v>156</v>
       </c>
       <c r="C105" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D105">
         <v>1</v>
@@ -2680,7 +2683,7 @@
         <v>160</v>
       </c>
       <c r="C106" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D106">
         <v>4</v>
@@ -2697,7 +2700,7 @@
         <v>165</v>
       </c>
       <c r="C107" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D107">
         <v>4</v>
@@ -2714,7 +2717,7 @@
         <v>180</v>
       </c>
       <c r="C108" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -2731,7 +2734,7 @@
         <v>181</v>
       </c>
       <c r="C109" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D109">
         <v>4</v>
@@ -2748,7 +2751,7 @@
         <v>182</v>
       </c>
       <c r="C110" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D110">
         <v>4</v>
@@ -2765,7 +2768,7 @@
         <v>183</v>
       </c>
       <c r="C111" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D111">
         <v>3</v>
@@ -2782,7 +2785,7 @@
         <v>184</v>
       </c>
       <c r="C112" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D112">
         <v>2</v>
@@ -2799,7 +2802,7 @@
         <v>185</v>
       </c>
       <c r="C113" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D113">
         <v>3</v>
@@ -2816,7 +2819,7 @@
         <v>186</v>
       </c>
       <c r="C114" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D114">
         <v>3</v>
@@ -2833,7 +2836,7 @@
         <v>187</v>
       </c>
       <c r="C115" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D115">
         <v>4</v>
@@ -2850,7 +2853,7 @@
         <v>188</v>
       </c>
       <c r="C116" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D116">
         <v>3</v>
@@ -2867,7 +2870,7 @@
         <v>189</v>
       </c>
       <c r="C117" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D117">
         <v>3</v>
@@ -2884,7 +2887,7 @@
         <v>190</v>
       </c>
       <c r="C118" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D118">
         <v>3</v>
@@ -2901,7 +2904,7 @@
         <v>191</v>
       </c>
       <c r="C119" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D119">
         <v>4</v>
@@ -2918,7 +2921,7 @@
         <v>198</v>
       </c>
       <c r="C120" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D120">
         <v>4</v>
@@ -2935,7 +2938,7 @@
         <v>199</v>
       </c>
       <c r="C121" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D121">
         <v>3</v>
@@ -2952,7 +2955,7 @@
         <v>200</v>
       </c>
       <c r="C122" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D122">
         <v>4</v>
@@ -2969,7 +2972,7 @@
         <v>201</v>
       </c>
       <c r="C123" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D123">
         <v>4</v>
@@ -2986,7 +2989,7 @@
         <v>202</v>
       </c>
       <c r="C124" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D124">
         <v>4</v>
@@ -3003,7 +3006,7 @@
         <v>203</v>
       </c>
       <c r="C125" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D125">
         <v>3</v>
@@ -3020,7 +3023,7 @@
         <v>204</v>
       </c>
       <c r="C126" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D126">
         <v>2</v>
@@ -3037,7 +3040,7 @@
         <v>205</v>
       </c>
       <c r="C127" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D127">
         <v>4</v>
@@ -3054,7 +3057,7 @@
         <v>206</v>
       </c>
       <c r="C128" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D128">
         <v>3</v>
@@ -3071,7 +3074,7 @@
         <v>207</v>
       </c>
       <c r="C129" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D129">
         <v>4</v>
@@ -3088,7 +3091,7 @@
         <v>208</v>
       </c>
       <c r="C130" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D130">
         <v>4</v>
@@ -3105,7 +3108,7 @@
         <v>209</v>
       </c>
       <c r="C131" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -3122,7 +3125,7 @@
         <v>210</v>
       </c>
       <c r="C132" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D132">
         <v>3</v>
@@ -3139,7 +3142,7 @@
         <v>211</v>
       </c>
       <c r="C133" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D133">
         <v>4</v>
@@ -3156,7 +3159,7 @@
         <v>212</v>
       </c>
       <c r="C134" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -3173,7 +3176,7 @@
         <v>213</v>
       </c>
       <c r="C135" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D135">
         <v>2</v>
@@ -3190,7 +3193,7 @@
         <v>214</v>
       </c>
       <c r="C136" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D136">
         <v>4</v>
@@ -3207,7 +3210,7 @@
         <v>215</v>
       </c>
       <c r="C137" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D137">
         <v>3</v>
@@ -3224,7 +3227,7 @@
         <v>216</v>
       </c>
       <c r="C138" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D138">
         <v>4</v>
@@ -3241,7 +3244,7 @@
         <v>217</v>
       </c>
       <c r="C139" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D139">
         <v>4</v>
@@ -3258,7 +3261,7 @@
         <v>218</v>
       </c>
       <c r="C140" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D140">
         <v>4</v>
@@ -3275,7 +3278,7 @@
         <v>219</v>
       </c>
       <c r="C141" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D141">
         <v>2</v>
@@ -3292,7 +3295,7 @@
         <v>220</v>
       </c>
       <c r="C142" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -3309,7 +3312,7 @@
         <v>221</v>
       </c>
       <c r="C143" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D143">
         <v>3</v>
@@ -3326,7 +3329,7 @@
         <v>222</v>
       </c>
       <c r="C144" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D144">
         <v>3</v>
@@ -3343,7 +3346,7 @@
         <v>223</v>
       </c>
       <c r="C145" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D145">
         <v>3</v>
@@ -3360,7 +3363,7 @@
         <v>224</v>
       </c>
       <c r="C146" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D146">
         <v>2</v>
@@ -3377,7 +3380,7 @@
         <v>225</v>
       </c>
       <c r="C147" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D147">
         <v>4</v>
@@ -3394,7 +3397,7 @@
         <v>226</v>
       </c>
       <c r="C148" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D148">
         <v>2</v>
@@ -3411,7 +3414,7 @@
         <v>227</v>
       </c>
       <c r="C149" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D149">
         <v>4</v>
@@ -3428,7 +3431,7 @@
         <v>228</v>
       </c>
       <c r="C150" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D150">
         <v>4</v>
@@ -3445,7 +3448,7 @@
         <v>229</v>
       </c>
       <c r="C151" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D151">
         <v>4</v>
@@ -3462,7 +3465,7 @@
         <v>230</v>
       </c>
       <c r="C152" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D152">
         <v>1</v>
@@ -3479,7 +3482,7 @@
         <v>231</v>
       </c>
       <c r="C153" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D153">
         <v>2</v>
@@ -3496,7 +3499,7 @@
         <v>232</v>
       </c>
       <c r="C154" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D154">
         <v>2</v>
@@ -3513,7 +3516,7 @@
         <v>233</v>
       </c>
       <c r="C155" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D155">
         <v>3</v>
@@ -3530,7 +3533,7 @@
         <v>234</v>
       </c>
       <c r="C156" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D156">
         <v>1</v>
@@ -3547,7 +3550,7 @@
         <v>235</v>
       </c>
       <c r="C157" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D157">
         <v>2</v>
@@ -3564,7 +3567,7 @@
         <v>236</v>
       </c>
       <c r="C158" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D158">
         <v>2</v>
@@ -3581,7 +3584,7 @@
         <v>237</v>
       </c>
       <c r="C159" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D159">
         <v>3</v>
@@ -3598,7 +3601,7 @@
         <v>238</v>
       </c>
       <c r="C160" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D160">
         <v>3</v>
@@ -3615,7 +3618,7 @@
         <v>239</v>
       </c>
       <c r="C161" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D161">
         <v>2</v>
@@ -3632,7 +3635,7 @@
         <v>240</v>
       </c>
       <c r="C162" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D162">
         <v>3</v>
@@ -3649,7 +3652,7 @@
         <v>241</v>
       </c>
       <c r="C163" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D163">
         <v>4</v>
@@ -3666,7 +3669,7 @@
         <v>242</v>
       </c>
       <c r="C164" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D164">
         <v>4</v>
@@ -3683,7 +3686,7 @@
         <v>243</v>
       </c>
       <c r="C165" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D165">
         <v>4</v>
@@ -3700,7 +3703,7 @@
         <v>244</v>
       </c>
       <c r="C166" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D166">
         <v>3</v>
@@ -3717,7 +3720,7 @@
         <v>245</v>
       </c>
       <c r="C167" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D167">
         <v>4</v>
@@ -3734,7 +3737,7 @@
         <v>246</v>
       </c>
       <c r="C168" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D168">
         <v>3</v>
@@ -3751,7 +3754,7 @@
         <v>247</v>
       </c>
       <c r="C169" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D169">
         <v>3</v>
@@ -3768,7 +3771,7 @@
         <v>248</v>
       </c>
       <c r="C170" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D170">
         <v>4</v>
@@ -3785,7 +3788,7 @@
         <v>249</v>
       </c>
       <c r="C171" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D171">
         <v>3</v>
@@ -3802,7 +3805,7 @@
         <v>250</v>
       </c>
       <c r="C172" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D172">
         <v>3</v>
@@ -3819,7 +3822,7 @@
         <v>251</v>
       </c>
       <c r="C173" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D173">
         <v>3</v>
@@ -3836,7 +3839,7 @@
         <v>252</v>
       </c>
       <c r="C174" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D174">
         <v>3</v>
@@ -3853,7 +3856,7 @@
         <v>253</v>
       </c>
       <c r="C175" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D175">
         <v>2</v>
@@ -3870,7 +3873,7 @@
         <v>254</v>
       </c>
       <c r="C176" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D176">
         <v>2</v>
@@ -3887,7 +3890,7 @@
         <v>255</v>
       </c>
       <c r="C177" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D177">
         <v>2</v>
@@ -3904,7 +3907,7 @@
         <v>256</v>
       </c>
       <c r="C178" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D178">
         <v>3</v>
@@ -3921,7 +3924,7 @@
         <v>257</v>
       </c>
       <c r="C179" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D179">
         <v>3</v>
@@ -3938,7 +3941,7 @@
         <v>258</v>
       </c>
       <c r="C180" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D180">
         <v>4</v>
@@ -3955,7 +3958,7 @@
         <v>259</v>
       </c>
       <c r="C181" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D181">
         <v>4</v>
@@ -3972,7 +3975,7 @@
         <v>260</v>
       </c>
       <c r="C182" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D182">
         <v>3</v>
@@ -3989,7 +3992,7 @@
         <v>261</v>
       </c>
       <c r="C183" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D183">
         <v>4</v>
@@ -4006,7 +4009,7 @@
         <v>262</v>
       </c>
       <c r="C184" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D184">
         <v>1</v>
@@ -4023,7 +4026,7 @@
         <v>263</v>
       </c>
       <c r="C185" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D185">
         <v>4</v>
@@ -4040,7 +4043,7 @@
         <v>264</v>
       </c>
       <c r="C186" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D186">
         <v>1</v>
@@ -4057,7 +4060,7 @@
         <v>265</v>
       </c>
       <c r="C187" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D187">
         <v>3</v>
@@ -4074,7 +4077,7 @@
         <v>266</v>
       </c>
       <c r="C188" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D188">
         <v>3</v>
@@ -4091,7 +4094,7 @@
         <v>267</v>
       </c>
       <c r="C189" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D189">
         <v>2</v>
@@ -4108,7 +4111,7 @@
         <v>268</v>
       </c>
       <c r="C190" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D190">
         <v>3</v>
@@ -4125,7 +4128,7 @@
         <v>269</v>
       </c>
       <c r="C191" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D191">
         <v>1</v>
@@ -4142,7 +4145,7 @@
         <v>270</v>
       </c>
       <c r="C192" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D192">
         <v>4</v>
@@ -4159,7 +4162,7 @@
         <v>271</v>
       </c>
       <c r="C193" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D193">
         <v>2</v>
@@ -4176,7 +4179,7 @@
         <v>272</v>
       </c>
       <c r="C194" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D194">
         <v>3</v>
@@ -4193,7 +4196,7 @@
         <v>273</v>
       </c>
       <c r="C195" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D195">
         <v>2</v>
@@ -4210,7 +4213,7 @@
         <v>274</v>
       </c>
       <c r="C196" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D196">
         <v>2</v>
@@ -4227,7 +4230,7 @@
         <v>275</v>
       </c>
       <c r="C197" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D197">
         <v>4</v>
@@ -4244,7 +4247,7 @@
         <v>276</v>
       </c>
       <c r="C198" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D198">
         <v>4</v>
@@ -4261,7 +4264,7 @@
         <v>277</v>
       </c>
       <c r="C199" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D199">
         <v>4</v>
@@ -4278,7 +4281,7 @@
         <v>278</v>
       </c>
       <c r="C200" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D200">
         <v>4</v>
@@ -4295,7 +4298,7 @@
         <v>279</v>
       </c>
       <c r="C201" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D201">
         <v>4</v>
@@ -4312,7 +4315,7 @@
         <v>280</v>
       </c>
       <c r="C202" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D202">
         <v>4</v>
@@ -4329,7 +4332,7 @@
         <v>281</v>
       </c>
       <c r="C203" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D203">
         <v>4</v>
@@ -4346,7 +4349,7 @@
         <v>282</v>
       </c>
       <c r="C204" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D204">
         <v>3</v>
@@ -4363,7 +4366,7 @@
         <v>283</v>
       </c>
       <c r="C205" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D205">
         <v>3</v>
@@ -4380,7 +4383,7 @@
         <v>284</v>
       </c>
       <c r="C206" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D206">
         <v>2</v>
@@ -4397,7 +4400,7 @@
         <v>285</v>
       </c>
       <c r="C207" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D207">
         <v>4</v>
@@ -4414,7 +4417,7 @@
         <v>286</v>
       </c>
       <c r="C208" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D208">
         <v>4</v>
@@ -4431,7 +4434,7 @@
         <v>287</v>
       </c>
       <c r="C209" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D209">
         <v>4</v>
@@ -4448,7 +4451,7 @@
         <v>288</v>
       </c>
       <c r="C210" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D210">
         <v>2</v>
@@ -4465,7 +4468,7 @@
         <v>289</v>
       </c>
       <c r="C211" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D211">
         <v>4</v>
@@ -4482,7 +4485,7 @@
         <v>290</v>
       </c>
       <c r="C212" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D212">
         <v>4</v>
@@ -4499,7 +4502,7 @@
         <v>291</v>
       </c>
       <c r="C213" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D213">
         <v>3</v>
@@ -4516,7 +4519,7 @@
         <v>292</v>
       </c>
       <c r="C214" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D214">
         <v>4</v>
@@ -4533,7 +4536,7 @@
         <v>293</v>
       </c>
       <c r="C215" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D215">
         <v>2</v>
@@ -4550,7 +4553,7 @@
         <v>294</v>
       </c>
       <c r="C216" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D216">
         <v>3</v>
@@ -4567,7 +4570,7 @@
         <v>295</v>
       </c>
       <c r="C217" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D217">
         <v>4</v>
@@ -4584,7 +4587,7 @@
         <v>296</v>
       </c>
       <c r="C218" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D218">
         <v>4</v>
@@ -4601,7 +4604,7 @@
         <v>297</v>
       </c>
       <c r="C219" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D219">
         <v>2</v>
@@ -4618,7 +4621,7 @@
         <v>298</v>
       </c>
       <c r="C220" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D220">
         <v>4</v>
@@ -4635,7 +4638,7 @@
         <v>299</v>
       </c>
       <c r="C221" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D221">
         <v>4</v>
@@ -4652,7 +4655,7 @@
         <v>300</v>
       </c>
       <c r="C222" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D222">
         <v>4</v>
@@ -4669,7 +4672,7 @@
         <v>301</v>
       </c>
       <c r="C223" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D223">
         <v>2</v>
@@ -4686,7 +4689,7 @@
         <v>302</v>
       </c>
       <c r="C224" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D224">
         <v>4</v>
@@ -4703,7 +4706,7 @@
         <v>303</v>
       </c>
       <c r="C225" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D225">
         <v>3</v>
@@ -4720,7 +4723,7 @@
         <v>304</v>
       </c>
       <c r="C226" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D226">
         <v>2</v>
@@ -4737,7 +4740,7 @@
         <v>305</v>
       </c>
       <c r="C227" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D227">
         <v>4</v>
@@ -4754,7 +4757,7 @@
         <v>306</v>
       </c>
       <c r="C228" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D228">
         <v>3</v>
@@ -4771,7 +4774,7 @@
         <v>307</v>
       </c>
       <c r="C229" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D229">
         <v>1</v>
@@ -4788,7 +4791,7 @@
         <v>308</v>
       </c>
       <c r="C230" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D230">
         <v>4</v>
@@ -4805,7 +4808,7 @@
         <v>309</v>
       </c>
       <c r="C231" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D231">
         <v>3</v>
@@ -4822,7 +4825,7 @@
         <v>310</v>
       </c>
       <c r="C232" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D232">
         <v>3</v>
@@ -4839,7 +4842,7 @@
         <v>311</v>
       </c>
       <c r="C233" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D233">
         <v>2</v>
@@ -4856,7 +4859,7 @@
         <v>312</v>
       </c>
       <c r="C234" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D234">
         <v>4</v>
@@ -4873,7 +4876,7 @@
         <v>313</v>
       </c>
       <c r="C235" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D235">
         <v>3</v>
@@ -4890,7 +4893,7 @@
         <v>314</v>
       </c>
       <c r="C236" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D236">
         <v>3</v>
@@ -4907,7 +4910,7 @@
         <v>315</v>
       </c>
       <c r="C237" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D237">
         <v>2</v>
@@ -4924,7 +4927,7 @@
         <v>316</v>
       </c>
       <c r="C238" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D238">
         <v>3</v>
@@ -4941,7 +4944,7 @@
         <v>317</v>
       </c>
       <c r="C239" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D239">
         <v>4</v>
@@ -4958,7 +4961,7 @@
         <v>318</v>
       </c>
       <c r="C240" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D240">
         <v>1</v>
@@ -4975,7 +4978,7 @@
         <v>319</v>
       </c>
       <c r="C241" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D241">
         <v>3</v>
@@ -4992,7 +4995,7 @@
         <v>320</v>
       </c>
       <c r="C242" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D242">
         <v>3</v>
@@ -5009,7 +5012,7 @@
         <v>321</v>
       </c>
       <c r="C243" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D243">
         <v>3</v>
@@ -5026,7 +5029,7 @@
         <v>322</v>
       </c>
       <c r="C244" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D244">
         <v>1</v>
@@ -5043,7 +5046,7 @@
         <v>323</v>
       </c>
       <c r="C245" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D245">
         <v>4</v>
@@ -5060,7 +5063,7 @@
         <v>324</v>
       </c>
       <c r="C246" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D246">
         <v>2</v>
@@ -5077,7 +5080,7 @@
         <v>325</v>
       </c>
       <c r="C247" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D247">
         <v>3</v>
@@ -5094,7 +5097,7 @@
         <v>326</v>
       </c>
       <c r="C248" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D248">
         <v>4</v>
@@ -5111,7 +5114,7 @@
         <v>327</v>
       </c>
       <c r="C249" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D249">
         <v>2</v>
@@ -5128,7 +5131,7 @@
         <v>328</v>
       </c>
       <c r="C250" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D250">
         <v>4</v>
@@ -5145,7 +5148,7 @@
         <v>329</v>
       </c>
       <c r="C251" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D251">
         <v>2</v>
@@ -5162,7 +5165,7 @@
         <v>330</v>
       </c>
       <c r="C252" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D252">
         <v>2</v>
@@ -5179,7 +5182,7 @@
         <v>331</v>
       </c>
       <c r="C253" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D253">
         <v>1</v>
@@ -5196,7 +5199,7 @@
         <v>332</v>
       </c>
       <c r="C254" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D254">
         <v>4</v>
@@ -5213,7 +5216,7 @@
         <v>333</v>
       </c>
       <c r="C255" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D255">
         <v>4</v>
@@ -5230,7 +5233,7 @@
         <v>334</v>
       </c>
       <c r="C256" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D256">
         <v>4</v>
@@ -5247,7 +5250,7 @@
         <v>335</v>
       </c>
       <c r="C257" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D257">
         <v>3</v>
@@ -5264,7 +5267,7 @@
         <v>336</v>
       </c>
       <c r="C258" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D258">
         <v>1</v>
@@ -5281,7 +5284,7 @@
         <v>337</v>
       </c>
       <c r="C259" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D259">
         <v>2</v>
@@ -5298,7 +5301,7 @@
         <v>338</v>
       </c>
       <c r="C260" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D260">
         <v>3</v>
@@ -5315,7 +5318,7 @@
         <v>339</v>
       </c>
       <c r="C261" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D261">
         <v>1</v>
@@ -5332,7 +5335,7 @@
         <v>340</v>
       </c>
       <c r="C262" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D262">
         <v>2</v>
@@ -5349,7 +5352,7 @@
         <v>341</v>
       </c>
       <c r="C263" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D263">
         <v>4</v>
@@ -5366,7 +5369,7 @@
         <v>342</v>
       </c>
       <c r="C264" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D264">
         <v>2</v>
@@ -5383,7 +5386,7 @@
         <v>343</v>
       </c>
       <c r="C265" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D265">
         <v>1</v>
@@ -5400,7 +5403,7 @@
         <v>344</v>
       </c>
       <c r="C266" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D266">
         <v>1</v>
@@ -5417,7 +5420,7 @@
         <v>345</v>
       </c>
       <c r="C267" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D267">
         <v>3</v>
@@ -5434,7 +5437,7 @@
         <v>346</v>
       </c>
       <c r="C268" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D268">
         <v>4</v>
@@ -5451,7 +5454,7 @@
         <v>347</v>
       </c>
       <c r="C269" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D269">
         <v>4</v>
@@ -5468,7 +5471,7 @@
         <v>348</v>
       </c>
       <c r="C270" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D270">
         <v>4</v>
@@ -5485,7 +5488,7 @@
         <v>349</v>
       </c>
       <c r="C271" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D271">
         <v>4</v>
@@ -5502,7 +5505,7 @@
         <v>350</v>
       </c>
       <c r="C272" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D272">
         <v>2</v>
@@ -5519,7 +5522,7 @@
         <v>351</v>
       </c>
       <c r="C273" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D273">
         <v>1</v>
@@ -5536,7 +5539,7 @@
         <v>352</v>
       </c>
       <c r="C274" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D274">
         <v>4</v>
@@ -5553,7 +5556,7 @@
         <v>353</v>
       </c>
       <c r="C275" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D275">
         <v>3</v>
@@ -5570,7 +5573,7 @@
         <v>354</v>
       </c>
       <c r="C276" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D276">
         <v>3</v>
@@ -5587,7 +5590,7 @@
         <v>355</v>
       </c>
       <c r="C277" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D277">
         <v>4</v>
@@ -5604,7 +5607,7 @@
         <v>356</v>
       </c>
       <c r="C278" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D278">
         <v>3</v>
@@ -5621,7 +5624,7 @@
         <v>357</v>
       </c>
       <c r="C279" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D279">
         <v>3</v>
@@ -5638,7 +5641,7 @@
         <v>358</v>
       </c>
       <c r="C280" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D280">
         <v>4</v>
@@ -5655,7 +5658,7 @@
         <v>359</v>
       </c>
       <c r="C281" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D281">
         <v>4</v>
@@ -5672,7 +5675,7 @@
         <v>360</v>
       </c>
       <c r="C282" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D282">
         <v>3</v>
@@ -5689,7 +5692,7 @@
         <v>361</v>
       </c>
       <c r="C283" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D283">
         <v>4</v>
@@ -5706,7 +5709,7 @@
         <v>362</v>
       </c>
       <c r="C284" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D284">
         <v>4</v>
@@ -5723,7 +5726,7 @@
         <v>363</v>
       </c>
       <c r="C285" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D285">
         <v>2</v>
@@ -5740,7 +5743,7 @@
         <v>364</v>
       </c>
       <c r="C286" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D286">
         <v>4</v>
@@ -5757,7 +5760,7 @@
         <v>365</v>
       </c>
       <c r="C287" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D287">
         <v>4</v>
@@ -5774,7 +5777,7 @@
         <v>366</v>
       </c>
       <c r="C288" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D288">
         <v>3</v>
@@ -5791,7 +5794,7 @@
         <v>367</v>
       </c>
       <c r="C289" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D289">
         <v>4</v>
@@ -5808,7 +5811,7 @@
         <v>368</v>
       </c>
       <c r="C290" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D290">
         <v>1</v>
@@ -5825,7 +5828,7 @@
         <v>369</v>
       </c>
       <c r="C291" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D291">
         <v>3</v>
@@ -5842,7 +5845,7 @@
         <v>370</v>
       </c>
       <c r="C292" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D292">
         <v>2</v>
@@ -5859,7 +5862,7 @@
         <v>371</v>
       </c>
       <c r="C293" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D293">
         <v>4</v>
@@ -5876,7 +5879,7 @@
         <v>372</v>
       </c>
       <c r="C294" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D294">
         <v>2</v>
@@ -5893,7 +5896,7 @@
         <v>373</v>
       </c>
       <c r="C295" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D295">
         <v>4</v>
@@ -5910,7 +5913,7 @@
         <v>374</v>
       </c>
       <c r="C296" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D296">
         <v>4</v>
@@ -5927,7 +5930,7 @@
         <v>375</v>
       </c>
       <c r="C297" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D297">
         <v>2</v>
@@ -5944,7 +5947,7 @@
         <v>376</v>
       </c>
       <c r="C298" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D298">
         <v>1</v>
@@ -5961,7 +5964,7 @@
         <v>377</v>
       </c>
       <c r="C299" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D299">
         <v>3</v>
@@ -5978,7 +5981,7 @@
         <v>378</v>
       </c>
       <c r="C300" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D300">
         <v>3</v>
@@ -5995,7 +5998,7 @@
         <v>379</v>
       </c>
       <c r="C301" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D301">
         <v>4</v>
@@ -6012,7 +6015,7 @@
         <v>380</v>
       </c>
       <c r="C302" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D302">
         <v>4</v>
@@ -6029,7 +6032,7 @@
         <v>381</v>
       </c>
       <c r="C303" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D303">
         <v>4</v>
@@ -6046,7 +6049,7 @@
         <v>382</v>
       </c>
       <c r="C304" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D304">
         <v>3</v>
@@ -6063,7 +6066,7 @@
         <v>383</v>
       </c>
       <c r="C305" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D305">
         <v>4</v>
@@ -6080,7 +6083,7 @@
         <v>384</v>
       </c>
       <c r="C306" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D306">
         <v>2</v>
@@ -6097,7 +6100,7 @@
         <v>385</v>
       </c>
       <c r="C307" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D307">
         <v>3</v>
@@ -6114,7 +6117,7 @@
         <v>386</v>
       </c>
       <c r="C308" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D308">
         <v>3</v>
@@ -6131,7 +6134,7 @@
         <v>387</v>
       </c>
       <c r="C309" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D309">
         <v>4</v>
@@ -6148,7 +6151,7 @@
         <v>388</v>
       </c>
       <c r="C310" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D310">
         <v>3</v>
@@ -6165,7 +6168,7 @@
         <v>389</v>
       </c>
       <c r="C311" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D311">
         <v>3</v>
@@ -6182,7 +6185,7 @@
         <v>390</v>
       </c>
       <c r="C312" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D312">
         <v>4</v>
@@ -6199,7 +6202,7 @@
         <v>391</v>
       </c>
       <c r="C313" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D313">
         <v>4</v>
@@ -6216,7 +6219,7 @@
         <v>392</v>
       </c>
       <c r="C314" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D314">
         <v>3</v>
@@ -6233,7 +6236,7 @@
         <v>393</v>
       </c>
       <c r="C315" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D315">
         <v>4</v>
@@ -6250,7 +6253,7 @@
         <v>394</v>
       </c>
       <c r="C316" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D316">
         <v>2</v>
@@ -6267,7 +6270,7 @@
         <v>395</v>
       </c>
       <c r="C317" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D317">
         <v>2</v>
@@ -6284,7 +6287,7 @@
         <v>396</v>
       </c>
       <c r="C318" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D318">
         <v>4</v>
@@ -6301,7 +6304,7 @@
         <v>397</v>
       </c>
       <c r="C319" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D319">
         <v>3</v>
@@ -6318,7 +6321,7 @@
         <v>398</v>
       </c>
       <c r="C320" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D320">
         <v>1</v>
@@ -6335,7 +6338,7 @@
         <v>399</v>
       </c>
       <c r="C321" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D321">
         <v>4</v>
@@ -6352,7 +6355,7 @@
         <v>400</v>
       </c>
       <c r="C322" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D322">
         <v>3</v>
@@ -6369,7 +6372,7 @@
         <v>401</v>
       </c>
       <c r="C323" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D323">
         <v>2</v>
@@ -6386,7 +6389,7 @@
         <v>402</v>
       </c>
       <c r="C324" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D324">
         <v>3</v>
@@ -6403,7 +6406,7 @@
         <v>403</v>
       </c>
       <c r="C325" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D325">
         <v>4</v>
@@ -6420,7 +6423,7 @@
         <v>404</v>
       </c>
       <c r="C326" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D326">
         <v>2</v>
@@ -6437,7 +6440,7 @@
         <v>405</v>
       </c>
       <c r="C327" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D327">
         <v>1</v>
@@ -6454,7 +6457,7 @@
         <v>406</v>
       </c>
       <c r="C328" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D328">
         <v>3</v>
@@ -6471,7 +6474,7 @@
         <v>407</v>
       </c>
       <c r="C329" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D329">
         <v>4</v>
@@ -6488,7 +6491,7 @@
         <v>408</v>
       </c>
       <c r="C330" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D330">
         <v>2</v>
@@ -6505,7 +6508,7 @@
         <v>409</v>
       </c>
       <c r="C331" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D331">
         <v>3</v>
@@ -6522,7 +6525,7 @@
         <v>410</v>
       </c>
       <c r="C332" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D332">
         <v>2</v>
@@ -6539,7 +6542,7 @@
         <v>411</v>
       </c>
       <c r="C333" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D333">
         <v>1</v>
@@ -6556,7 +6559,7 @@
         <v>412</v>
       </c>
       <c r="C334" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D334">
         <v>3</v>
@@ -6573,7 +6576,7 @@
         <v>413</v>
       </c>
       <c r="C335" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D335">
         <v>4</v>
@@ -6590,7 +6593,7 @@
         <v>414</v>
       </c>
       <c r="C336" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D336">
         <v>4</v>
@@ -6607,7 +6610,7 @@
         <v>415</v>
       </c>
       <c r="C337" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D337">
         <v>4</v>
@@ -6624,7 +6627,7 @@
         <v>416</v>
       </c>
       <c r="C338" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D338">
         <v>2</v>
@@ -6641,7 +6644,7 @@
         <v>417</v>
       </c>
       <c r="C339" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D339">
         <v>2</v>
@@ -6658,7 +6661,7 @@
         <v>418</v>
       </c>
       <c r="C340" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D340">
         <v>4</v>
@@ -6675,7 +6678,7 @@
         <v>420</v>
       </c>
       <c r="C341" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D341">
         <v>3</v>
@@ -6692,7 +6695,7 @@
         <v>421</v>
       </c>
       <c r="C342" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D342">
         <v>4</v>
@@ -6709,7 +6712,7 @@
         <v>422</v>
       </c>
       <c r="C343" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D343">
         <v>4</v>
@@ -6726,7 +6729,7 @@
         <v>423</v>
       </c>
       <c r="C344" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D344">
         <v>3</v>
@@ -6743,7 +6746,7 @@
         <v>424</v>
       </c>
       <c r="C345" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D345">
         <v>3</v>
@@ -6760,7 +6763,7 @@
         <v>425</v>
       </c>
       <c r="C346" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D346">
         <v>4</v>
@@ -6777,7 +6780,7 @@
         <v>426</v>
       </c>
       <c r="C347" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D347">
         <v>4</v>
@@ -6794,7 +6797,7 @@
         <v>427</v>
       </c>
       <c r="C348" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D348">
         <v>1</v>
@@ -6811,7 +6814,7 @@
         <v>428</v>
       </c>
       <c r="C349" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D349">
         <v>3</v>
@@ -6828,7 +6831,7 @@
         <v>429</v>
       </c>
       <c r="C350" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D350">
         <v>1</v>
@@ -6845,7 +6848,7 @@
         <v>430</v>
       </c>
       <c r="C351" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D351">
         <v>4</v>
@@ -6862,7 +6865,7 @@
         <v>431</v>
       </c>
       <c r="C352" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D352">
         <v>2</v>
@@ -6879,7 +6882,7 @@
         <v>432</v>
       </c>
       <c r="C353" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D353">
         <v>3</v>
@@ -6896,7 +6899,7 @@
         <v>433</v>
       </c>
       <c r="C354" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D354">
         <v>3</v>
@@ -6913,7 +6916,7 @@
         <v>434</v>
       </c>
       <c r="C355" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D355">
         <v>4</v>
@@ -6930,7 +6933,7 @@
         <v>435</v>
       </c>
       <c r="C356" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D356">
         <v>2</v>
@@ -6947,7 +6950,7 @@
         <v>436</v>
       </c>
       <c r="C357" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D357">
         <v>4</v>
@@ -6964,7 +6967,7 @@
         <v>437</v>
       </c>
       <c r="C358" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D358">
         <v>3</v>
@@ -6981,7 +6984,7 @@
         <v>438</v>
       </c>
       <c r="C359" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D359">
         <v>4</v>
@@ -6998,7 +7001,7 @@
         <v>439</v>
       </c>
       <c r="C360" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D360">
         <v>4</v>
@@ -7015,7 +7018,7 @@
         <v>440</v>
       </c>
       <c r="C361" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D361">
         <v>2</v>
@@ -7032,7 +7035,7 @@
         <v>441</v>
       </c>
       <c r="C362" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D362">
         <v>2</v>
@@ -7049,7 +7052,7 @@
         <v>442</v>
       </c>
       <c r="C363" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D363">
         <v>4</v>
@@ -7066,7 +7069,7 @@
         <v>443</v>
       </c>
       <c r="C364" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D364">
         <v>1</v>
@@ -7083,7 +7086,7 @@
         <v>444</v>
       </c>
       <c r="C365" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D365">
         <v>4</v>
@@ -7100,7 +7103,7 @@
         <v>445</v>
       </c>
       <c r="C366" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D366">
         <v>4</v>
@@ -7117,7 +7120,7 @@
         <v>446</v>
       </c>
       <c r="C367" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D367">
         <v>4</v>
@@ -7134,7 +7137,7 @@
         <v>447</v>
       </c>
       <c r="C368" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D368">
         <v>3</v>
@@ -7151,7 +7154,7 @@
         <v>448</v>
       </c>
       <c r="C369" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D369">
         <v>2</v>
@@ -7168,7 +7171,7 @@
         <v>449</v>
       </c>
       <c r="C370" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D370">
         <v>3</v>
@@ -7185,7 +7188,7 @@
         <v>450</v>
       </c>
       <c r="C371" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D371">
         <v>3</v>

</xml_diff>